<commit_message>
feat: run rate logic
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -931,7 +931,7 @@
         <v>Amey</v>
       </c>
       <c r="C6">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
@@ -942,7 +942,7 @@
         <v>Mala</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -953,7 +953,7 @@
         <v>Siddharth</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -964,7 +964,7 @@
         <v>Supriya</v>
       </c>
       <c r="C9">
-        <v>42</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -1604,7 +1604,7 @@
         <v>Home - News</v>
       </c>
       <c r="D41" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="42">
@@ -1618,7 +1618,7 @@
         <v>Home - Videos</v>
       </c>
       <c r="D42" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="43">
@@ -1632,7 +1632,7 @@
         <v>Points Table</v>
       </c>
       <c r="D43" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="44">
@@ -1646,7 +1646,7 @@
         <v>Stats</v>
       </c>
       <c r="D44" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="45">
@@ -1660,7 +1660,7 @@
         <v>Showcase</v>
       </c>
       <c r="D45" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="46">
@@ -1702,7 +1702,7 @@
         <v>Home - Fixtures</v>
       </c>
       <c r="D48" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="49">
@@ -1716,7 +1716,7 @@
         <v>Header &amp; Footer, Sponsors</v>
       </c>
       <c r="D49" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="50">
@@ -1730,7 +1730,7 @@
         <v>Home - Players</v>
       </c>
       <c r="D50" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="51">
@@ -1744,7 +1744,7 @@
         <v>FREE Due Blocker</v>
       </c>
       <c r="D51" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="52">
@@ -1758,7 +1758,7 @@
         <v>Wf fixses</v>
       </c>
       <c r="D52" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="53">
@@ -1800,7 +1800,7 @@
         <v>player Profile</v>
       </c>
       <c r="D55" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="56">
@@ -1814,7 +1814,7 @@
         <v>Fixses</v>
       </c>
       <c r="D56" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="57">
@@ -1828,7 +1828,7 @@
         <v>Support</v>
       </c>
       <c r="D57" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="58">
@@ -1842,7 +1842,7 @@
         <v>GO Live</v>
       </c>
       <c r="D58" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="59">
@@ -1856,7 +1856,7 @@
         <v>Top Menu, Bottom Menu</v>
       </c>
       <c r="D59" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="60">
@@ -1870,7 +1870,7 @@
         <v>Footer</v>
       </c>
       <c r="D60" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="61">
@@ -1884,7 +1884,7 @@
         <v>Both Standings css</v>
       </c>
       <c r="D61" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="62">
@@ -1898,7 +1898,7 @@
         <v>HP News</v>
       </c>
       <c r="D62" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="63">
@@ -1912,7 +1912,7 @@
         <v>HP Videos</v>
       </c>
       <c r="D63" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="64">
@@ -1926,7 +1926,7 @@
         <v>HP Photos</v>
       </c>
       <c r="D64" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="65">
@@ -1940,7 +1940,7 @@
         <v>News Listing &amp; Detail</v>
       </c>
       <c r="D65" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="66">
@@ -1954,7 +1954,7 @@
         <v>Video Listing and Detail</v>
       </c>
       <c r="D66" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="67">
@@ -1968,7 +1968,7 @@
         <v>Photos Listing &amp; Detail</v>
       </c>
       <c r="D67" t="str">
-        <v>done</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="68">
@@ -1996,7 +1996,7 @@
         <v>Privacy Policy</v>
       </c>
       <c r="D69" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="70">
@@ -2010,7 +2010,7 @@
         <v>Thank you</v>
       </c>
       <c r="D70" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="71">
@@ -2024,7 +2024,7 @@
         <v>404</v>
       </c>
       <c r="D71" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="72">
@@ -2038,7 +2038,7 @@
         <v>Partnership Framework</v>
       </c>
       <c r="D72" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="73">
@@ -2052,7 +2052,7 @@
         <v>Where to Watch</v>
       </c>
       <c r="D73" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="74">
@@ -2066,7 +2066,7 @@
         <v>Womens t20 exhibition</v>
       </c>
       <c r="D74" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="75">
@@ -2080,7 +2080,7 @@
         <v>Wallpapers</v>
       </c>
       <c r="D75" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="76">
@@ -2122,7 +2122,7 @@
         <v>Boundary Builder page + form</v>
       </c>
       <c r="D78" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="79">
@@ -2136,7 +2136,7 @@
         <v>Unit testing fixses of all form</v>
       </c>
       <c r="D79" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="80">
@@ -2150,7 +2150,7 @@
         <v>Videos - Listing</v>
       </c>
       <c r="D80" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="81">
@@ -2164,7 +2164,7 @@
         <v>Photos - Listing</v>
       </c>
       <c r="D81" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="82">
@@ -2178,7 +2178,7 @@
         <v>News - Listing</v>
       </c>
       <c r="D82" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="83">
@@ -2192,7 +2192,7 @@
         <v>Photos - Detail</v>
       </c>
       <c r="D83" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="84">
@@ -2206,7 +2206,7 @@
         <v>News - Detail</v>
       </c>
       <c r="D84" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="85">
@@ -2220,7 +2220,7 @@
         <v>Videos - Detail</v>
       </c>
       <c r="D85" t="str">
-        <v>inprogress</v>
+        <v>done</v>
       </c>
     </row>
     <row r="86">
@@ -2234,7 +2234,7 @@
         <v>Showcase</v>
       </c>
       <c r="D86" t="str">
-        <v>inprogress</v>
+        <v>pending</v>
       </c>
     </row>
     <row r="87">

</xml_diff>

<commit_message>
Sync task checklist statuses from Jira, add apply-jira-statuses workflow
Corrects 30 task rows (WF/SO) where the sheet's Status was stale vs.
the actual Jira ticket status. Adds scripts/apply-jira-statuses.mjs so
this can be re-run by feeding it a {TaskID: status} map pulled via
Claude's connected Jira access, rather than requiring an API token in
sync-from-sheet.mjs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -488,88 +488,88 @@
     <t>Home - News</t>
   </si>
   <si>
+    <t>FNS-101</t>
+  </si>
+  <si>
+    <t>Home - Videos</t>
+  </si>
+  <si>
+    <t>2026-08-11</t>
+  </si>
+  <si>
+    <t>FNS-51</t>
+  </si>
+  <si>
+    <t>Points Table</t>
+  </si>
+  <si>
+    <t>FNS-49</t>
+  </si>
+  <si>
+    <t>Stats</t>
+  </si>
+  <si>
+    <t>FNS-6</t>
+  </si>
+  <si>
+    <t>Showcase</t>
+  </si>
+  <si>
+    <t>2026-08-12</t>
+  </si>
+  <si>
+    <t>FNS-13</t>
+  </si>
+  <si>
+    <t>Home - shop</t>
+  </si>
+  <si>
+    <t>2026-08-13</t>
+  </si>
+  <si>
+    <t>FNS-41</t>
+  </si>
+  <si>
+    <t>Schedule</t>
+  </si>
+  <si>
+    <t>2026-08-26</t>
+  </si>
+  <si>
+    <t>FNS-8</t>
+  </si>
+  <si>
+    <t>Home - Fixtures</t>
+  </si>
+  <si>
+    <t>2026-08-14</t>
+  </si>
+  <si>
+    <t>FNS-5</t>
+  </si>
+  <si>
+    <t>Header &amp; Footer, Sponsors</t>
+  </si>
+  <si>
+    <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>FNS-12</t>
+  </si>
+  <si>
+    <t>Home - Players</t>
+  </si>
+  <si>
+    <t>2026-08-18</t>
+  </si>
+  <si>
+    <t>2026-08-19</t>
+  </si>
+  <si>
+    <t>FREE Due Blocker</t>
+  </si>
+  <si>
     <t>pending</t>
-  </si>
-  <si>
-    <t>FNS-101</t>
-  </si>
-  <si>
-    <t>Home - Videos</t>
-  </si>
-  <si>
-    <t>2026-08-11</t>
-  </si>
-  <si>
-    <t>FNS-51</t>
-  </si>
-  <si>
-    <t>Points Table</t>
-  </si>
-  <si>
-    <t>FNS-49</t>
-  </si>
-  <si>
-    <t>Stats</t>
-  </si>
-  <si>
-    <t>FNS-6</t>
-  </si>
-  <si>
-    <t>Showcase</t>
-  </si>
-  <si>
-    <t>2026-08-12</t>
-  </si>
-  <si>
-    <t>FNS-13</t>
-  </si>
-  <si>
-    <t>Home - shop</t>
-  </si>
-  <si>
-    <t>2026-08-13</t>
-  </si>
-  <si>
-    <t>FNS-41</t>
-  </si>
-  <si>
-    <t>Schedule</t>
-  </si>
-  <si>
-    <t>2026-08-26</t>
-  </si>
-  <si>
-    <t>FNS-8</t>
-  </si>
-  <si>
-    <t>Home - Fixtures</t>
-  </si>
-  <si>
-    <t>2026-08-14</t>
-  </si>
-  <si>
-    <t>FNS-5</t>
-  </si>
-  <si>
-    <t>Header &amp; Footer, Sponsors</t>
-  </si>
-  <si>
-    <t>2026-08-17</t>
-  </si>
-  <si>
-    <t>FNS-12</t>
-  </si>
-  <si>
-    <t>Home - Players</t>
-  </si>
-  <si>
-    <t>2026-08-18</t>
-  </si>
-  <si>
-    <t>2026-08-19</t>
-  </si>
-  <si>
-    <t>FREE Due Blocker</t>
   </si>
   <si>
     <t>Wf fixses</t>
@@ -1535,7 +1535,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1871,7 +1871,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2036,7 +2036,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2046,7 +2046,7 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3109,7 +3109,7 @@
         <v>39</v>
       </c>
       <c r="G28" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H28" t="s">
         <v>39</v>
@@ -4495,206 +4495,206 @@
         <v>75</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="263" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="264" spans="4:4" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid date" error="Please enter a valid date." sqref="A10:A264">
@@ -4791,7 +4791,7 @@
     <hyperlink ref="D64" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <tableParts count="1">
     <tablePart r:id="rId63"/>
   </tableParts>
@@ -4869,7 +4869,7 @@
         <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
         <v>39</v>
@@ -4898,16 +4898,16 @@
         <v>40</v>
       </c>
       <c r="D3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" t="s">
         <v>157</v>
       </c>
-      <c r="E3" t="s">
-        <v>158</v>
-      </c>
       <c r="F3" t="s">
         <v>39</v>
       </c>
       <c r="G3" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
         <v>39</v>
@@ -4927,7 +4927,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -4936,10 +4936,10 @@
         <v>40</v>
       </c>
       <c r="D4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E4" t="s">
         <v>160</v>
-      </c>
-      <c r="E4" t="s">
-        <v>161</v>
       </c>
       <c r="F4" t="s">
         <v>39</v>
@@ -4951,10 +4951,10 @@
         <v>39</v>
       </c>
       <c r="I4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -4965,7 +4965,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -4974,25 +4974,25 @@
         <v>40</v>
       </c>
       <c r="D5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E5" t="s">
         <v>162</v>
       </c>
-      <c r="E5" t="s">
-        <v>163</v>
-      </c>
       <c r="F5" t="s">
         <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H5" t="s">
         <v>39</v>
       </c>
       <c r="I5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J5" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K5" t="s">
         <v>39</v>
@@ -5003,7 +5003,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -5012,25 +5012,25 @@
         <v>40</v>
       </c>
       <c r="D6" t="s">
+        <v>163</v>
+      </c>
+      <c r="E6" t="s">
         <v>164</v>
       </c>
-      <c r="E6" t="s">
-        <v>165</v>
-      </c>
       <c r="F6" t="s">
         <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
         <v>39</v>
       </c>
       <c r="I6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="J6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K6" t="s">
         <v>39</v>
@@ -5041,7 +5041,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -5050,36 +5050,36 @@
         <v>40</v>
       </c>
       <c r="D7" t="s">
+        <v>166</v>
+      </c>
+      <c r="E7" t="s">
         <v>167</v>
       </c>
-      <c r="E7" t="s">
-        <v>168</v>
-      </c>
       <c r="F7" t="s">
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H7" t="s">
         <v>39</v>
       </c>
       <c r="I7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K7" t="s">
         <v>39</v>
       </c>
       <c r="L7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B8" t="s">
         <v>2</v>
@@ -5088,10 +5088,10 @@
         <v>40</v>
       </c>
       <c r="D8" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" t="s">
         <v>170</v>
-      </c>
-      <c r="E8" t="s">
-        <v>171</v>
       </c>
       <c r="F8" t="s">
         <v>39</v>
@@ -5103,10 +5103,10 @@
         <v>39</v>
       </c>
       <c r="I8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J8" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K8" t="s">
         <v>39</v>
@@ -5117,7 +5117,7 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B9" t="s">
         <v>2</v>
@@ -5126,25 +5126,25 @@
         <v>40</v>
       </c>
       <c r="D9" t="s">
+        <v>172</v>
+      </c>
+      <c r="E9" t="s">
         <v>173</v>
       </c>
-      <c r="E9" t="s">
-        <v>174</v>
-      </c>
       <c r="F9" t="s">
         <v>39</v>
       </c>
       <c r="G9" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H9" t="s">
         <v>39</v>
       </c>
       <c r="I9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K9" t="s">
         <v>39</v>
@@ -5155,7 +5155,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B10" t="s">
         <v>2</v>
@@ -5164,25 +5164,25 @@
         <v>40</v>
       </c>
       <c r="D10" t="s">
+        <v>175</v>
+      </c>
+      <c r="E10" t="s">
         <v>176</v>
       </c>
-      <c r="E10" t="s">
-        <v>177</v>
-      </c>
       <c r="F10" t="s">
         <v>39</v>
       </c>
       <c r="G10" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H10" t="s">
         <v>39</v>
       </c>
       <c r="I10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="J10" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K10" t="s">
         <v>39</v>
@@ -5193,7 +5193,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
@@ -5202,22 +5202,22 @@
         <v>40</v>
       </c>
       <c r="D11" t="s">
+        <v>178</v>
+      </c>
+      <c r="E11" t="s">
         <v>179</v>
       </c>
-      <c r="E11" t="s">
-        <v>180</v>
-      </c>
       <c r="F11" t="s">
         <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H11" t="s">
         <v>39</v>
       </c>
       <c r="I11" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J11" t="s">
         <v>38</v>
@@ -5231,7 +5231,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B12" t="s">
         <v>2</v>
@@ -5240,22 +5240,22 @@
         <v>40</v>
       </c>
       <c r="D12" t="s">
+        <v>178</v>
+      </c>
+      <c r="E12" t="s">
         <v>179</v>
       </c>
-      <c r="E12" t="s">
-        <v>180</v>
-      </c>
       <c r="F12" t="s">
         <v>39</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H12" t="s">
         <v>39</v>
       </c>
       <c r="I12" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J12" t="s">
         <v>38</v>
@@ -5269,7 +5269,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B13" t="s">
         <v>2</v>
@@ -5281,22 +5281,22 @@
         <v>39</v>
       </c>
       <c r="E13" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" t="s">
         <v>183</v>
       </c>
-      <c r="F13" t="s">
-        <v>39</v>
-      </c>
-      <c r="G13" t="s">
-        <v>156</v>
-      </c>
       <c r="H13" t="s">
         <v>39</v>
       </c>
       <c r="I13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K13" t="s">
         <v>39</v>
@@ -5325,7 +5325,7 @@
         <v>39</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H14" t="s">
         <v>39</v>
@@ -5354,22 +5354,22 @@
         <v>40</v>
       </c>
       <c r="D15" t="s">
+        <v>178</v>
+      </c>
+      <c r="E15" t="s">
         <v>179</v>
       </c>
-      <c r="E15" t="s">
-        <v>180</v>
-      </c>
       <c r="F15" t="s">
         <v>39</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H15" t="s">
         <v>39</v>
       </c>
       <c r="I15" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J15" t="s">
         <v>38</v>
@@ -5392,10 +5392,10 @@
         <v>40</v>
       </c>
       <c r="D16" t="s">
+        <v>169</v>
+      </c>
+      <c r="E16" t="s">
         <v>170</v>
-      </c>
-      <c r="E16" t="s">
-        <v>171</v>
       </c>
       <c r="F16" t="s">
         <v>39</v>
@@ -5407,10 +5407,10 @@
         <v>39</v>
       </c>
       <c r="I16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J16" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K16" t="s">
         <v>39</v>
@@ -5506,10 +5506,10 @@
         <v>40</v>
       </c>
       <c r="D19" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" t="s">
         <v>170</v>
-      </c>
-      <c r="E19" t="s">
-        <v>171</v>
       </c>
       <c r="F19" t="s">
         <v>39</v>
@@ -5521,10 +5521,10 @@
         <v>39</v>
       </c>
       <c r="I19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J19" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K19" t="s">
         <v>39</v>
@@ -5535,7 +5535,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B20" t="s">
         <v>2</v>
@@ -5544,10 +5544,10 @@
         <v>40</v>
       </c>
       <c r="D20" t="s">
+        <v>169</v>
+      </c>
+      <c r="E20" t="s">
         <v>170</v>
-      </c>
-      <c r="E20" t="s">
-        <v>171</v>
       </c>
       <c r="F20" t="s">
         <v>39</v>
@@ -5559,10 +5559,10 @@
         <v>39</v>
       </c>
       <c r="I20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K20" t="s">
         <v>39</v>
@@ -5573,7 +5573,7 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B21" t="s">
         <v>2</v>
@@ -5597,10 +5597,10 @@
         <v>39</v>
       </c>
       <c r="I21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K21" t="s">
         <v>39</v>
@@ -5629,7 +5629,7 @@
         <v>39</v>
       </c>
       <c r="G22" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H22" t="s">
         <v>39</v>
@@ -5667,7 +5667,7 @@
         <v>39</v>
       </c>
       <c r="G23" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H23" t="s">
         <v>39</v>
@@ -5705,7 +5705,7 @@
         <v>39</v>
       </c>
       <c r="G24" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H24" t="s">
         <v>39</v>
@@ -5743,7 +5743,7 @@
         <v>39</v>
       </c>
       <c r="G25" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H25" t="s">
         <v>39</v>
@@ -5781,7 +5781,7 @@
         <v>39</v>
       </c>
       <c r="G26" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H26" t="s">
         <v>39</v>
@@ -5819,7 +5819,7 @@
         <v>39</v>
       </c>
       <c r="G27" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H27" t="s">
         <v>39</v>
@@ -5857,7 +5857,7 @@
         <v>39</v>
       </c>
       <c r="G28" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H28" t="s">
         <v>39</v>
@@ -5895,7 +5895,7 @@
         <v>39</v>
       </c>
       <c r="G29" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H29" t="s">
         <v>39</v>
@@ -5933,7 +5933,7 @@
         <v>39</v>
       </c>
       <c r="G30" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
         <v>39</v>
@@ -6047,7 +6047,7 @@
         <v>39</v>
       </c>
       <c r="G33" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H33" t="s">
         <v>39</v>
@@ -6085,7 +6085,7 @@
         <v>39</v>
       </c>
       <c r="G34" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H34" t="s">
         <v>39</v>
@@ -6123,7 +6123,7 @@
         <v>39</v>
       </c>
       <c r="G35" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H35" t="s">
         <v>39</v>
@@ -6161,7 +6161,7 @@
         <v>39</v>
       </c>
       <c r="G36" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H36" t="s">
         <v>39</v>
@@ -6199,7 +6199,7 @@
         <v>39</v>
       </c>
       <c r="G37" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H37" t="s">
         <v>39</v>
@@ -6237,7 +6237,7 @@
         <v>39</v>
       </c>
       <c r="G38" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H38" t="s">
         <v>39</v>
@@ -6257,7 +6257,7 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B39" t="s">
         <v>6</v>
@@ -6275,16 +6275,16 @@
         <v>39</v>
       </c>
       <c r="G39" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H39" t="s">
         <v>39</v>
       </c>
       <c r="I39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J39" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K39" t="s">
         <v>39</v>
@@ -6295,7 +6295,7 @@
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B40" t="s">
         <v>6</v>
@@ -6313,16 +6313,16 @@
         <v>39</v>
       </c>
       <c r="G40" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H40" t="s">
         <v>39</v>
       </c>
       <c r="I40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J40" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K40" t="s">
         <v>39</v>
@@ -6351,7 +6351,7 @@
         <v>39</v>
       </c>
       <c r="G41" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H41" t="s">
         <v>39</v>
@@ -6389,7 +6389,7 @@
         <v>39</v>
       </c>
       <c r="G42" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H42" t="s">
         <v>39</v>
@@ -6427,7 +6427,7 @@
         <v>39</v>
       </c>
       <c r="G43" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H43" t="s">
         <v>39</v>
@@ -6465,7 +6465,7 @@
         <v>39</v>
       </c>
       <c r="G44" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H44" t="s">
         <v>39</v>
@@ -6541,7 +6541,7 @@
         <v>39</v>
       </c>
       <c r="G46" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H46" t="s">
         <v>39</v>
@@ -6617,7 +6617,7 @@
         <v>39</v>
       </c>
       <c r="G48" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H48" t="s">
         <v>39</v>
@@ -6637,7 +6637,7 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B49" t="s">
         <v>9</v>
@@ -6655,16 +6655,16 @@
         <v>39</v>
       </c>
       <c r="G49" t="s">
-        <v>156</v>
+        <v>44</v>
       </c>
       <c r="H49" t="s">
         <v>39</v>
       </c>
       <c r="I49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J49" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K49" t="s">
         <v>39</v>
@@ -6693,7 +6693,7 @@
         <v>39</v>
       </c>
       <c r="G50" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H50" t="s">
         <v>39</v>
@@ -6713,7 +6713,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B51" t="s">
         <v>10</v>
@@ -6731,16 +6731,16 @@
         <v>39</v>
       </c>
       <c r="G51" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H51" t="s">
         <v>39</v>
       </c>
       <c r="I51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J51" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K51" t="s">
         <v>39</v>
@@ -6751,7 +6751,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B52" t="s">
         <v>10</v>
@@ -6769,16 +6769,16 @@
         <v>39</v>
       </c>
       <c r="G52" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H52" t="s">
         <v>39</v>
       </c>
       <c r="I52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K52" t="s">
         <v>39</v>
@@ -6789,7 +6789,7 @@
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B53" t="s">
         <v>10</v>
@@ -6807,16 +6807,16 @@
         <v>39</v>
       </c>
       <c r="G53" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H53" t="s">
         <v>39</v>
       </c>
       <c r="I53" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J53" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K53" t="s">
         <v>39</v>
@@ -6827,7 +6827,7 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B54" t="s">
         <v>10</v>
@@ -6845,16 +6845,16 @@
         <v>39</v>
       </c>
       <c r="G54" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H54" t="s">
         <v>39</v>
       </c>
       <c r="I54" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J54" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K54" t="s">
         <v>39</v>
@@ -6865,7 +6865,7 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B55" t="s">
         <v>10</v>
@@ -6883,16 +6883,16 @@
         <v>39</v>
       </c>
       <c r="G55" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H55" t="s">
         <v>39</v>
       </c>
       <c r="I55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K55" t="s">
         <v>39</v>
@@ -6921,7 +6921,7 @@
         <v>39</v>
       </c>
       <c r="G56" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H56" t="s">
         <v>39</v>
@@ -6959,7 +6959,7 @@
         <v>39</v>
       </c>
       <c r="G57" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H57" t="s">
         <v>39</v>
@@ -6997,7 +6997,7 @@
         <v>39</v>
       </c>
       <c r="G58" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="H58" t="s">
         <v>39</v>
@@ -7029,7 +7029,7 @@
         <v>39</v>
       </c>
       <c r="E59" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F59" t="s">
         <v>39</v>
@@ -7093,7 +7093,7 @@
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B61" t="s">
         <v>10</v>
@@ -7167,206 +7167,206 @@
         <v>39</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="253" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="254" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="255" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="256" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="257" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="258" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="259" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="260" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="261" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="262" spans="4:4" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid date" error="Please enter a valid date." sqref="A10:A262">
@@ -7443,7 +7443,7 @@
     <hyperlink ref="D62" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <tableParts count="1">
     <tablePart r:id="rId43"/>
   </tableParts>
@@ -7521,7 +7521,7 @@
         <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H2" t="s">
         <v>39</v>
@@ -7559,7 +7559,7 @@
         <v>39</v>
       </c>
       <c r="G3" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H3" t="s">
         <v>39</v>
@@ -7597,7 +7597,7 @@
         <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H4" t="s">
         <v>39</v>
@@ -7635,7 +7635,7 @@
         <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
         <v>39</v>
@@ -7673,7 +7673,7 @@
         <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H6" t="s">
         <v>39</v>
@@ -7711,7 +7711,7 @@
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H7" t="s">
         <v>39</v>
@@ -7749,7 +7749,7 @@
         <v>39</v>
       </c>
       <c r="G8" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H8" t="s">
         <v>39</v>
@@ -7787,7 +7787,7 @@
         <v>39</v>
       </c>
       <c r="G9" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H9" t="s">
         <v>39</v>
@@ -7825,7 +7825,7 @@
         <v>39</v>
       </c>
       <c r="G10" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H10" t="s">
         <v>39</v>
@@ -7863,7 +7863,7 @@
         <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H11" t="s">
         <v>39</v>
@@ -7901,7 +7901,7 @@
         <v>39</v>
       </c>
       <c r="G12" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H12" t="s">
         <v>39</v>
@@ -7939,7 +7939,7 @@
         <v>39</v>
       </c>
       <c r="G13" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H13" t="s">
         <v>39</v>
@@ -7977,7 +7977,7 @@
         <v>39</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H14" t="s">
         <v>39</v>
@@ -8015,7 +8015,7 @@
         <v>39</v>
       </c>
       <c r="G15" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H15" t="s">
         <v>39</v>
@@ -8053,7 +8053,7 @@
         <v>39</v>
       </c>
       <c r="G16" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H16" t="s">
         <v>39</v>
@@ -8091,7 +8091,7 @@
         <v>39</v>
       </c>
       <c r="G17" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H17" t="s">
         <v>39</v>
@@ -8129,7 +8129,7 @@
         <v>39</v>
       </c>
       <c r="G18" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H18" t="s">
         <v>39</v>
@@ -8167,7 +8167,7 @@
         <v>39</v>
       </c>
       <c r="G19" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H19" t="s">
         <v>39</v>
@@ -8205,7 +8205,7 @@
         <v>39</v>
       </c>
       <c r="G20" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H20" t="s">
         <v>39</v>
@@ -8243,7 +8243,7 @@
         <v>39</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H21" t="s">
         <v>39</v>
@@ -8281,7 +8281,7 @@
         <v>39</v>
       </c>
       <c r="G22" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H22" t="s">
         <v>39</v>
@@ -8319,7 +8319,7 @@
         <v>39</v>
       </c>
       <c r="G23" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H23" t="s">
         <v>39</v>
@@ -8357,7 +8357,7 @@
         <v>39</v>
       </c>
       <c r="G24" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H24" t="s">
         <v>39</v>
@@ -8395,7 +8395,7 @@
         <v>39</v>
       </c>
       <c r="G25" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H25" t="s">
         <v>39</v>
@@ -8433,7 +8433,7 @@
         <v>39</v>
       </c>
       <c r="G26" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H26" t="s">
         <v>39</v>
@@ -8471,7 +8471,7 @@
         <v>39</v>
       </c>
       <c r="G27" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H27" t="s">
         <v>39</v>
@@ -8509,7 +8509,7 @@
         <v>39</v>
       </c>
       <c r="G28" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H28" t="s">
         <v>39</v>
@@ -8547,7 +8547,7 @@
         <v>39</v>
       </c>
       <c r="G29" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H29" t="s">
         <v>39</v>
@@ -8585,7 +8585,7 @@
         <v>39</v>
       </c>
       <c r="G30" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
         <v>39</v>
@@ -8623,7 +8623,7 @@
         <v>39</v>
       </c>
       <c r="G31" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H31" t="s">
         <v>39</v>
@@ -8661,7 +8661,7 @@
         <v>39</v>
       </c>
       <c r="G32" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H32" t="s">
         <v>39</v>
@@ -8699,7 +8699,7 @@
         <v>39</v>
       </c>
       <c r="G33" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H33" t="s">
         <v>39</v>
@@ -8737,7 +8737,7 @@
         <v>39</v>
       </c>
       <c r="G34" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H34" t="s">
         <v>39</v>
@@ -8775,7 +8775,7 @@
         <v>39</v>
       </c>
       <c r="G35" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H35" t="s">
         <v>39</v>
@@ -8813,7 +8813,7 @@
         <v>39</v>
       </c>
       <c r="G36" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H36" t="s">
         <v>39</v>
@@ -8851,7 +8851,7 @@
         <v>39</v>
       </c>
       <c r="G37" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H37" t="s">
         <v>39</v>
@@ -8889,7 +8889,7 @@
         <v>39</v>
       </c>
       <c r="G38" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H38" t="s">
         <v>39</v>
@@ -8927,7 +8927,7 @@
         <v>39</v>
       </c>
       <c r="G39" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H39" t="s">
         <v>39</v>
@@ -8945,206 +8945,206 @@
         <v>39</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="4:4" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid date" error="Please enter a valid date." sqref="A10:A239">
@@ -9177,7 +9177,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -9255,7 +9255,7 @@
         <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H2" t="s">
         <v>39</v>
@@ -9293,7 +9293,7 @@
         <v>39</v>
       </c>
       <c r="G3" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H3" t="s">
         <v>39</v>
@@ -9331,7 +9331,7 @@
         <v>39</v>
       </c>
       <c r="G4" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H4" t="s">
         <v>39</v>
@@ -9369,7 +9369,7 @@
         <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
         <v>39</v>
@@ -9407,7 +9407,7 @@
         <v>39</v>
       </c>
       <c r="G6" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H6" t="s">
         <v>39</v>
@@ -9445,7 +9445,7 @@
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H7" t="s">
         <v>39</v>
@@ -9483,7 +9483,7 @@
         <v>39</v>
       </c>
       <c r="G8" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H8" t="s">
         <v>39</v>
@@ -9556,7 +9556,7 @@
         <v>39</v>
       </c>
       <c r="G10" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H10" t="s">
         <v>39</v>
@@ -9588,13 +9588,13 @@
         <v>39</v>
       </c>
       <c r="E11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F11" t="s">
         <v>39</v>
       </c>
       <c r="G11" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H11" t="s">
         <v>39</v>
@@ -9632,7 +9632,7 @@
         <v>39</v>
       </c>
       <c r="G12" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H12" t="s">
         <v>39</v>
@@ -9670,7 +9670,7 @@
         <v>39</v>
       </c>
       <c r="G13" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H13" t="s">
         <v>39</v>
@@ -9708,7 +9708,7 @@
         <v>-0.5</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H14" t="s">
         <v>39</v>
@@ -9746,7 +9746,7 @@
         <v>39</v>
       </c>
       <c r="G15" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H15" t="s">
         <v>39</v>
@@ -9784,7 +9784,7 @@
         <v>39</v>
       </c>
       <c r="G16" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H16" t="s">
         <v>39</v>
@@ -9822,7 +9822,7 @@
         <v>-0.5</v>
       </c>
       <c r="G17" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H17" t="s">
         <v>39</v>
@@ -9860,7 +9860,7 @@
         <v>39</v>
       </c>
       <c r="G18" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H18" t="s">
         <v>39</v>
@@ -9898,7 +9898,7 @@
         <v>39</v>
       </c>
       <c r="G19" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H19" t="s">
         <v>39</v>
@@ -9936,7 +9936,7 @@
         <v>39</v>
       </c>
       <c r="G20" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H20" t="s">
         <v>39</v>
@@ -9974,7 +9974,7 @@
         <v>39</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H21" t="s">
         <v>39</v>
@@ -10012,7 +10012,7 @@
         <v>39</v>
       </c>
       <c r="G22" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H22" t="s">
         <v>39</v>
@@ -10050,7 +10050,7 @@
         <v>-6</v>
       </c>
       <c r="G23" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H23" t="s">
         <v>39</v>
@@ -10088,7 +10088,7 @@
         <v>39</v>
       </c>
       <c r="G24" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H24" t="s">
         <v>39</v>
@@ -10126,7 +10126,7 @@
         <v>39</v>
       </c>
       <c r="G25" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H25" t="s">
         <v>39</v>
@@ -10164,7 +10164,7 @@
         <v>39</v>
       </c>
       <c r="G26" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H26" t="s">
         <v>39</v>
@@ -10202,7 +10202,7 @@
         <v>39</v>
       </c>
       <c r="G27" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H27" t="s">
         <v>39</v>
@@ -10240,7 +10240,7 @@
         <v>39</v>
       </c>
       <c r="G28" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H28" t="s">
         <v>39</v>
@@ -10278,7 +10278,7 @@
         <v>39</v>
       </c>
       <c r="G29" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H29" t="s">
         <v>39</v>
@@ -10316,7 +10316,7 @@
         <v>39</v>
       </c>
       <c r="G30" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H30" t="s">
         <v>39</v>
@@ -10354,7 +10354,7 @@
         <v>39</v>
       </c>
       <c r="G31" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H31" t="s">
         <v>39</v>
@@ -10392,7 +10392,7 @@
         <v>39</v>
       </c>
       <c r="G32" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H32" t="s">
         <v>39</v>
@@ -10430,7 +10430,7 @@
         <v>39</v>
       </c>
       <c r="G33" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H33" t="s">
         <v>39</v>
@@ -10468,7 +10468,7 @@
         <v>-4</v>
       </c>
       <c r="G34" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H34" t="s">
         <v>39</v>
@@ -10506,7 +10506,7 @@
         <v>-4</v>
       </c>
       <c r="G35" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H35" t="s">
         <v>39</v>
@@ -10544,7 +10544,7 @@
         <v>-2</v>
       </c>
       <c r="G36" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H36" t="s">
         <v>39</v>
@@ -10582,7 +10582,7 @@
         <v>-2</v>
       </c>
       <c r="G37" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H37" t="s">
         <v>39</v>
@@ -10620,7 +10620,7 @@
         <v>-2</v>
       </c>
       <c r="G38" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H38" t="s">
         <v>39</v>
@@ -10658,7 +10658,7 @@
         <v>-4</v>
       </c>
       <c r="G39" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H39" t="s">
         <v>39</v>
@@ -10696,7 +10696,7 @@
         <v>-2</v>
       </c>
       <c r="G40" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H40" t="s">
         <v>39</v>
@@ -10734,7 +10734,7 @@
         <v>-2</v>
       </c>
       <c r="G41" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H41" t="s">
         <v>39</v>
@@ -10772,7 +10772,7 @@
         <v>-4</v>
       </c>
       <c r="G42" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H42" t="s">
         <v>39</v>
@@ -10810,7 +10810,7 @@
         <v>39</v>
       </c>
       <c r="G43" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H43" t="s">
         <v>39</v>
@@ -10848,7 +10848,7 @@
         <v>39</v>
       </c>
       <c r="G44" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H44" t="s">
         <v>39</v>
@@ -10886,7 +10886,7 @@
         <v>39</v>
       </c>
       <c r="G45" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H45" t="s">
         <v>39</v>
@@ -10924,7 +10924,7 @@
         <v>39</v>
       </c>
       <c r="G46" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H46" t="s">
         <v>39</v>
@@ -10962,7 +10962,7 @@
         <v>39</v>
       </c>
       <c r="G47" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H47" t="s">
         <v>39</v>
@@ -11000,7 +11000,7 @@
         <v>39</v>
       </c>
       <c r="G48" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H48" t="s">
         <v>39</v>
@@ -11038,7 +11038,7 @@
         <v>39</v>
       </c>
       <c r="G49" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H49" t="s">
         <v>39</v>
@@ -11076,7 +11076,7 @@
         <v>39</v>
       </c>
       <c r="G50" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H50" t="s">
         <v>39</v>
@@ -11114,7 +11114,7 @@
         <v>39</v>
       </c>
       <c r="G51" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H51" t="s">
         <v>39</v>
@@ -11152,7 +11152,7 @@
         <v>39</v>
       </c>
       <c r="G52" t="s">
-        <v>156</v>
+        <v>183</v>
       </c>
       <c r="H52" t="s">
         <v>39</v>
@@ -11170,206 +11170,206 @@
         <v>39</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="75" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="76" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="77" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="78" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="79" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="80" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="81" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="82" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="107" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="108" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="109" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="110" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="111" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="112" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="113" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="114" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="115" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="116" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="117" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="119" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="120" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="121" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="122" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="123" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="124" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="125" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="126" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="127" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="128" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="129" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="130" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="131" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="132" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="133" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="134" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="135" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="136" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="137" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="139" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="140" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="142" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="143" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="144" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="145" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="146" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="147" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="148" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="149" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="150" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="151" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="152" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="161" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="162" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="163" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="164" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="165" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="166" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="167" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="168" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="169" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="170" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="171" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="173" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="174" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="175" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="176" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="177" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="178" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="179" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="180" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="181" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="182" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="183" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="184" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="185" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="193" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="194" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="195" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="196" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="197" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="198" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="199" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="200" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="201" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="202" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="203" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="204" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="205" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="206" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="207" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="208" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="209" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="210" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="211" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="212" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="213" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="214" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="215" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="216" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="217" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="218" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="219" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="220" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="221" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="222" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="223" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="224" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="225" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="226" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="227" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="228" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="229" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="230" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="231" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="232" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="233" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="234" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="235" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="236" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="237" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="238" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="239" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="240" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="241" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="242" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="243" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="244" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="245" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="246" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="247" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="248" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="249" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="250" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="251" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="252" spans="4:4" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid date" error="Please enter a valid date." sqref="A10:A252">
@@ -11402,7 +11402,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Fix Siddharth name mismatch hiding the Innings Split section
"Siddharth N" (used in PVL/MCFC log entries) didn't match "Siddharth"
in the Developers sheet, so that developer's team lookup came back NA
— which hid the whole Home/Away Innings Split (it requires every squad
member to have a resolved team). Renamed to "Siddharth" in both
sheets so their hours roll up under the one developer entry.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2622" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2622" uniqueCount="308">
   <si>
     <t>Name</t>
   </si>
@@ -801,9 +801,6 @@
   </si>
   <si>
     <t>Error Page</t>
-  </si>
-  <si>
-    <t>Siddharth N</t>
   </si>
   <si>
     <t>Header &amp; Footer</t>
@@ -4780,7 +4777,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M262"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5288,7 +5285,6 @@
         <v>160</v>
       </c>
     </row>
-    <row r="14" spans="5:5" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>38</v>
@@ -5617,11 +5613,6 @@
         <v>196</v>
       </c>
     </row>
-    <row r="23" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="5:5" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>197</v>
@@ -6518,15 +6509,6 @@
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>189</v>
@@ -6688,206 +6670,6 @@
         <v>215</v>
       </c>
     </row>
-    <row r="63" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="5:5" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="5:5" x14ac:dyDescent="0.25"/>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="Invalid date" error="Please enter a valid date." sqref="A10:A262">
@@ -7791,7 +7573,7 @@
         <v>225</v>
       </c>
       <c r="B22" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C22" t="s">
         <v>45</v>
@@ -7800,7 +7582,7 @@
         <v>39</v>
       </c>
       <c r="E22" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F22" t="s">
         <v>39</v>
@@ -7829,7 +7611,7 @@
         <v>240</v>
       </c>
       <c r="B23" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C23" t="s">
         <v>45</v>
@@ -7838,7 +7620,7 @@
         <v>39</v>
       </c>
       <c r="E23" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F23" t="s">
         <v>39</v>
@@ -7876,7 +7658,7 @@
         <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F24" t="s">
         <v>39</v>
@@ -7914,7 +7696,7 @@
         <v>39</v>
       </c>
       <c r="E25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F25" t="s">
         <v>39</v>
@@ -7952,7 +7734,7 @@
         <v>39</v>
       </c>
       <c r="E26" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F26" t="s">
         <v>39</v>
@@ -7981,7 +7763,7 @@
         <v>43</v>
       </c>
       <c r="B27" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C27" t="s">
         <v>45</v>
@@ -7990,7 +7772,7 @@
         <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F27" t="s">
         <v>39</v>
@@ -8019,7 +7801,7 @@
         <v>197</v>
       </c>
       <c r="B28" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C28" t="s">
         <v>45</v>
@@ -8028,7 +7810,7 @@
         <v>39</v>
       </c>
       <c r="E28" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F28" t="s">
         <v>39</v>
@@ -8057,7 +7839,7 @@
         <v>201</v>
       </c>
       <c r="B29" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C29" t="s">
         <v>45</v>
@@ -8066,7 +7848,7 @@
         <v>39</v>
       </c>
       <c r="E29" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F29" t="s">
         <v>39</v>
@@ -8095,7 +7877,7 @@
         <v>204</v>
       </c>
       <c r="B30" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C30" t="s">
         <v>45</v>
@@ -8104,7 +7886,7 @@
         <v>39</v>
       </c>
       <c r="E30" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F30" t="s">
         <v>39</v>
@@ -8133,7 +7915,7 @@
         <v>163</v>
       </c>
       <c r="B31" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C31" t="s">
         <v>45</v>
@@ -8171,7 +7953,7 @@
         <v>184</v>
       </c>
       <c r="B32" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C32" t="s">
         <v>45</v>
@@ -8180,7 +7962,7 @@
         <v>39</v>
       </c>
       <c r="E32" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F32" t="s">
         <v>39</v>
@@ -8209,7 +7991,7 @@
         <v>184</v>
       </c>
       <c r="B33" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C33" t="s">
         <v>45</v>
@@ -8218,7 +8000,7 @@
         <v>39</v>
       </c>
       <c r="E33" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F33" t="s">
         <v>39</v>
@@ -8256,7 +8038,7 @@
         <v>39</v>
       </c>
       <c r="E34" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F34" t="s">
         <v>39</v>
@@ -8294,7 +8076,7 @@
         <v>39</v>
       </c>
       <c r="E35" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F35" t="s">
         <v>39</v>
@@ -8332,7 +8114,7 @@
         <v>39</v>
       </c>
       <c r="E36" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F36" t="s">
         <v>39</v>
@@ -8370,7 +8152,7 @@
         <v>39</v>
       </c>
       <c r="E37" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F37" t="s">
         <v>39</v>
@@ -8399,7 +8181,7 @@
         <v>248</v>
       </c>
       <c r="B38" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C38" t="s">
         <v>45</v>
@@ -8408,7 +8190,7 @@
         <v>39</v>
       </c>
       <c r="E38" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F38" t="s">
         <v>39</v>
@@ -8446,7 +8228,7 @@
         <v>39</v>
       </c>
       <c r="E39" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F39" t="s">
         <v>39</v>
@@ -8565,7 +8347,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -8577,7 +8359,7 @@
         <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F2" t="s">
         <v>39</v>
@@ -8589,10 +8371,10 @@
         <v>39</v>
       </c>
       <c r="I2" t="s">
+        <v>274</v>
+      </c>
+      <c r="J2" t="s">
         <v>275</v>
-      </c>
-      <c r="J2" t="s">
-        <v>276</v>
       </c>
       <c r="K2" t="s">
         <v>39</v>
@@ -8603,7 +8385,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
@@ -8615,7 +8397,7 @@
         <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F3" t="s">
         <v>39</v>
@@ -8627,10 +8409,10 @@
         <v>39</v>
       </c>
       <c r="I3" t="s">
+        <v>274</v>
+      </c>
+      <c r="J3" t="s">
         <v>275</v>
-      </c>
-      <c r="J3" t="s">
-        <v>276</v>
       </c>
       <c r="K3" t="s">
         <v>39</v>
@@ -8641,7 +8423,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -8653,7 +8435,7 @@
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F4" t="s">
         <v>39</v>
@@ -8665,10 +8447,10 @@
         <v>39</v>
       </c>
       <c r="I4" t="s">
+        <v>274</v>
+      </c>
+      <c r="J4" t="s">
         <v>275</v>
-      </c>
-      <c r="J4" t="s">
-        <v>276</v>
       </c>
       <c r="K4" t="s">
         <v>39</v>
@@ -8679,7 +8461,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
@@ -8691,7 +8473,7 @@
         <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F5" t="s">
         <v>39</v>
@@ -8703,10 +8485,10 @@
         <v>39</v>
       </c>
       <c r="I5" t="s">
+        <v>274</v>
+      </c>
+      <c r="J5" t="s">
         <v>275</v>
-      </c>
-      <c r="J5" t="s">
-        <v>276</v>
       </c>
       <c r="K5" t="s">
         <v>39</v>
@@ -8717,7 +8499,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -8729,7 +8511,7 @@
         <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F6" t="s">
         <v>39</v>
@@ -8741,10 +8523,10 @@
         <v>39</v>
       </c>
       <c r="I6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K6" t="s">
         <v>39</v>
@@ -8755,7 +8537,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -8767,7 +8549,7 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F7" t="s">
         <v>39</v>
@@ -8779,10 +8561,10 @@
         <v>39</v>
       </c>
       <c r="I7" t="s">
+        <v>274</v>
+      </c>
+      <c r="J7" t="s">
         <v>275</v>
-      </c>
-      <c r="J7" t="s">
-        <v>276</v>
       </c>
       <c r="K7" t="s">
         <v>39</v>
@@ -8793,7 +8575,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -8805,7 +8587,7 @@
         <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F8" t="s">
         <v>39</v>
@@ -8817,10 +8599,10 @@
         <v>39</v>
       </c>
       <c r="I8" t="s">
+        <v>274</v>
+      </c>
+      <c r="J8" t="s">
         <v>275</v>
-      </c>
-      <c r="J8" t="s">
-        <v>276</v>
       </c>
       <c r="K8" t="s">
         <v>39</v>
@@ -8840,7 +8622,7 @@
         <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F9" t="s">
         <v>39</v>
@@ -8878,7 +8660,7 @@
         <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F10" t="s">
         <v>39</v>
@@ -8904,7 +8686,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B11" t="s">
         <v>6</v>
@@ -8928,10 +8710,10 @@
         <v>39</v>
       </c>
       <c r="I11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J11" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K11" t="s">
         <v>39</v>
@@ -8942,7 +8724,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B12" t="s">
         <v>8</v>
@@ -8954,7 +8736,7 @@
         <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F12" t="s">
         <v>39</v>
@@ -8966,7 +8748,7 @@
         <v>39</v>
       </c>
       <c r="I12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J12" t="s">
         <v>43</v>
@@ -8992,7 +8774,7 @@
         <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F13" t="s">
         <v>39</v>
@@ -9068,7 +8850,7 @@
         <v>39</v>
       </c>
       <c r="E15" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F15" t="s">
         <v>39</v>
@@ -9094,10 +8876,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B16" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
@@ -9106,7 +8888,7 @@
         <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F16" t="s">
         <v>39</v>
@@ -9118,10 +8900,10 @@
         <v>39</v>
       </c>
       <c r="I16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J16" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K16" t="s">
         <v>39</v>
@@ -9182,7 +8964,7 @@
         <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F18" t="s">
         <v>39</v>
@@ -9211,7 +8993,7 @@
         <v>49</v>
       </c>
       <c r="B19" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C19" t="s">
         <v>51</v>
@@ -9220,7 +9002,7 @@
         <v>39</v>
       </c>
       <c r="E19" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F19" t="s">
         <v>39</v>
@@ -9235,7 +9017,7 @@
         <v>49</v>
       </c>
       <c r="J19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K19" t="s">
         <v>39</v>
@@ -9246,7 +9028,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B20" t="s">
         <v>6</v>
@@ -9258,7 +9040,7 @@
         <v>39</v>
       </c>
       <c r="E20" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F20" t="s">
         <v>39</v>
@@ -9270,10 +9052,10 @@
         <v>39</v>
       </c>
       <c r="I20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J20" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K20" t="s">
         <v>39</v>
@@ -9296,7 +9078,7 @@
         <v>39</v>
       </c>
       <c r="E21" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F21" t="s">
         <v>39</v>
@@ -9334,7 +9116,7 @@
         <v>39</v>
       </c>
       <c r="E22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F22" t="s">
         <v>39</v>
@@ -9349,7 +9131,7 @@
         <v>43</v>
       </c>
       <c r="J22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="K22" t="s">
         <v>39</v>
@@ -9410,7 +9192,7 @@
         <v>39</v>
       </c>
       <c r="E24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F24" t="s">
         <v>39</v>
@@ -9448,7 +9230,7 @@
         <v>39</v>
       </c>
       <c r="E25" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F25" t="s">
         <v>39</v>
@@ -9486,7 +9268,7 @@
         <v>39</v>
       </c>
       <c r="E26" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F26" t="s">
         <v>39</v>
@@ -9524,7 +9306,7 @@
         <v>39</v>
       </c>
       <c r="E27" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F27" t="s">
         <v>39</v>
@@ -9562,7 +9344,7 @@
         <v>39</v>
       </c>
       <c r="E28" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F28" t="s">
         <v>39</v>
@@ -9588,7 +9370,7 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B29" t="s">
         <v>6</v>
@@ -9600,7 +9382,7 @@
         <v>39</v>
       </c>
       <c r="E29" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F29" t="s">
         <v>39</v>
@@ -9612,10 +9394,10 @@
         <v>39</v>
       </c>
       <c r="I29" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K29" t="s">
         <v>39</v>
@@ -9676,7 +9458,7 @@
         <v>39</v>
       </c>
       <c r="E31" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F31" t="s">
         <v>39</v>
@@ -9702,7 +9484,7 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B32" t="s">
         <v>8</v>
@@ -9714,7 +9496,7 @@
         <v>39</v>
       </c>
       <c r="E32" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F32" t="s">
         <v>39</v>
@@ -9726,7 +9508,7 @@
         <v>39</v>
       </c>
       <c r="I32" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J32" t="s">
         <v>43</v>
@@ -10120,10 +9902,10 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B43" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C43" t="s">
         <v>51</v>
@@ -10132,7 +9914,7 @@
         <v>39</v>
       </c>
       <c r="E43" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F43" t="s">
         <v>39</v>
@@ -10144,10 +9926,10 @@
         <v>39</v>
       </c>
       <c r="I43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J43" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K43" t="s">
         <v>39</v>
@@ -10158,10 +9940,10 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B44" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C44" t="s">
         <v>51</v>
@@ -10170,7 +9952,7 @@
         <v>39</v>
       </c>
       <c r="E44" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F44" t="s">
         <v>39</v>
@@ -10182,10 +9964,10 @@
         <v>39</v>
       </c>
       <c r="I44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="K44" t="s">
         <v>39</v>
@@ -10196,10 +9978,10 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B45" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
@@ -10208,7 +9990,7 @@
         <v>39</v>
       </c>
       <c r="E45" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F45" t="s">
         <v>39</v>
@@ -10220,10 +10002,10 @@
         <v>39</v>
       </c>
       <c r="I45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J45" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K45" t="s">
         <v>39</v>
@@ -10234,10 +10016,10 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B46" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C46" t="s">
         <v>51</v>
@@ -10246,7 +10028,7 @@
         <v>39</v>
       </c>
       <c r="E46" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F46" t="s">
         <v>39</v>
@@ -10258,10 +10040,10 @@
         <v>39</v>
       </c>
       <c r="I46" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J46" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K46" t="s">
         <v>39</v>
@@ -10272,10 +10054,10 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B47" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C47" t="s">
         <v>51</v>
@@ -10284,7 +10066,7 @@
         <v>39</v>
       </c>
       <c r="E47" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F47" t="s">
         <v>39</v>
@@ -10296,10 +10078,10 @@
         <v>39</v>
       </c>
       <c r="I47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="K47" t="s">
         <v>39</v>
@@ -10310,10 +10092,10 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B48" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C48" t="s">
         <v>51</v>
@@ -10322,7 +10104,7 @@
         <v>39</v>
       </c>
       <c r="E48" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F48" t="s">
         <v>39</v>
@@ -10334,10 +10116,10 @@
         <v>39</v>
       </c>
       <c r="I48" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J48" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="K48" t="s">
         <v>39</v>
@@ -10348,10 +10130,10 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B49" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C49" t="s">
         <v>51</v>
@@ -10360,7 +10142,7 @@
         <v>39</v>
       </c>
       <c r="E49" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F49" t="s">
         <v>39</v>
@@ -10372,10 +10154,10 @@
         <v>39</v>
       </c>
       <c r="I49" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="J49" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="K49" t="s">
         <v>39</v>
@@ -10386,10 +10168,10 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B50" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C50" t="s">
         <v>51</v>
@@ -10398,7 +10180,7 @@
         <v>39</v>
       </c>
       <c r="E50" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="F50" t="s">
         <v>39</v>
@@ -10410,10 +10192,10 @@
         <v>39</v>
       </c>
       <c r="I50" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J50" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K50" t="s">
         <v>39</v>
@@ -10424,10 +10206,10 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B51" t="s">
-        <v>261</v>
+        <v>9</v>
       </c>
       <c r="C51" t="s">
         <v>51</v>
@@ -10436,7 +10218,7 @@
         <v>39</v>
       </c>
       <c r="E51" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="F51" t="s">
         <v>39</v>
@@ -10448,10 +10230,10 @@
         <v>39</v>
       </c>
       <c r="I51" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J51" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="K51" t="s">
         <v>39</v>
@@ -10474,7 +10256,7 @@
         <v>39</v>
       </c>
       <c r="E52" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F52" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
Consolidate Jira status + hours sync into one script/command
Replaces apply-jira-statuses.mjs with scripts/sync-dashboard.mjs,
which takes one payload (statuses, hours, newTasks, newDevelopers —
any section optional) and applies all of it to FML-Data.xlsx in a
single write, then regenerates generated.json once. "Ask Claude to
update the dashboard" now covers ticket statuses, hours, and any new
tasks/developers in one request instead of asking for each separately.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -5955,6 +5955,9 @@
         <v>105</v>
       </c>
     </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>219</v>
@@ -6851,6 +6854,15 @@
         <v>204</v>
       </c>
     </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>207</v>

</xml_diff>

<commit_message>
Add manual hours override: Shubham 61h on WF
Shubham had no Jira worklog entries, so the worklog-derived
HoursOverride replace dropped him to 0h. Adding back as a manual
override for hours worked that weren't logged against a ticket.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2719" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="331">
   <si>
     <t>Name</t>
   </si>
@@ -2002,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2146,6 +2146,17 @@
       </c>
       <c r="C13">
         <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add manual hours override: Mayur 32h on WF
SO's 8h (from a Jira worklog on a Rejected ticket) stays as-is; this
is a separate WF override for hours worked that weren't logged
against a ticket.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="331">
   <si>
     <t>Name</t>
   </si>
@@ -2002,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2157,6 +2157,17 @@
       </c>
       <c r="C14">
         <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh dashboard from latest Jira data
Ticket statuses unchanged since last sync. Hours refreshed: Suraj R.
Chavan's SO worklog total grew to 20.8h, and Mayur's SO 8h dropped to
0 since that ticket's (FNS-48) worklog entry was deleted in Jira.
Manual WF overrides (Shubham 61h, Mayur 32h) preserved.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2723" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="331">
   <si>
     <t>Name</t>
   </si>
@@ -2002,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -2046,7 +2046,7 @@
         <v>13</v>
       </c>
       <c r="C4">
-        <v>17.1</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2076,21 +2076,21 @@
         <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C8">
-        <v>56</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2098,10 +2098,10 @@
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C9">
-        <v>35</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2109,10 +2109,10 @@
         <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C10">
-        <v>66</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2120,10 +2120,10 @@
         <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="C11">
-        <v>15.8</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -2131,10 +2131,10 @@
         <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="C12">
-        <v>47</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -2142,10 +2142,10 @@
         <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C13">
-        <v>30</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2153,20 +2153,9 @@
         <v>40</v>
       </c>
       <c r="B14" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C14">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15">
         <v>32</v>
       </c>
     </row>
@@ -6019,6 +6008,9 @@
         <v>108</v>
       </c>
     </row>
+    <row r="25" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>222</v>
@@ -6915,6 +6907,15 @@
         <v>207</v>
       </c>
     </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="52" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="4:4" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>210</v>

</xml_diff>

<commit_message>
Distribute +40h proportionally into SO's dev+QA planned split
Planned_BuildDev/RunDev/QA (the budget Required RR is actually scoped
to) increase by 40h total, split proportionally to their existing
values (52/152/40 -> 60.5/176.9/46.6), so Required RR now reflects
the same +40h bump already applied to TargetHours.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/data/FML-Data.xlsx
+++ b/src/data/FML-Data.xlsx
@@ -1974,19 +1974,19 @@
         <v>52</v>
       </c>
       <c r="J3">
-        <v>52</v>
+        <v>60.5</v>
       </c>
       <c r="K3">
         <v>50</v>
       </c>
       <c r="L3">
-        <v>152</v>
+        <v>176.9</v>
       </c>
       <c r="M3">
         <v>80</v>
       </c>
       <c r="N3">
-        <v>40</v>
+        <v>46.6</v>
       </c>
       <c r="O3">
         <v>24</v>

</xml_diff>